<commit_message>
Try and preempt row height for text being translated
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/06-producer-certificate-start.xlsx
+++ b/translations/welsh-translations/06-producer-certificate-start.xlsx
@@ -658,7 +658,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -878,7 +878,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>

</xml_diff>